<commit_message>
feat: IIP and CPI from the MoSPI API (base-spliced), FY27 fiscal deficit BE, drop superseded raw/interim files; 53 modelling rows to Q1 FY27; docs updated
</commit_message>
<xml_diff>
--- a/data/processed/composite_master_quarterly.xlsx
+++ b/data/processed/composite_master_quarterly.xlsx
@@ -1022,7 +1022,7 @@
         <v>8.5</v>
       </c>
       <c r="K5" t="n">
-        <v>7.78</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -1055,7 +1055,7 @@
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="n">
-        <v>0.7199999999999998</v>
+        <v>-0.1199999999999992</v>
       </c>
       <c r="AE5" t="n">
         <v>5957.187441333333</v>
@@ -1137,7 +1137,7 @@
         <v>8.088888888888889</v>
       </c>
       <c r="K6" t="n">
-        <v>9.903333333333334</v>
+        <v>10.18333333333333</v>
       </c>
       <c r="L6" t="n">
         <v>2.2</v>
@@ -1180,7 +1180,7 @@
         <v>15.82326235219023</v>
       </c>
       <c r="AD6" t="n">
-        <v>-1.814444444444446</v>
+        <v>-2.094444444444443</v>
       </c>
       <c r="AE6" t="n">
         <v>5865.912661111111</v>
@@ -1192,7 +1192,7 @@
         <v>15.82326235219023</v>
       </c>
       <c r="AH6" t="n">
-        <v>5.919929018856893</v>
+        <v>5.639929018856895</v>
       </c>
       <c r="AI6" t="n">
         <v>2072727.7</v>
@@ -1270,7 +1270,7 @@
         <v>8</v>
       </c>
       <c r="K7" t="n">
-        <v>10.02666666666667</v>
+        <v>9.873333333333333</v>
       </c>
       <c r="L7" t="n">
         <v>0.1333333333333333</v>
@@ -1313,7 +1313,7 @@
         <v>13.63341342336888</v>
       </c>
       <c r="AD7" t="n">
-        <v>-2.026666666666666</v>
+        <v>-1.873333333333333</v>
       </c>
       <c r="AE7" t="n">
         <v>6052.851920444445</v>
@@ -1325,7 +1325,7 @@
         <v>13.63341342336888</v>
       </c>
       <c r="AH7" t="n">
-        <v>3.606746756702213</v>
+        <v>3.760080090035546</v>
       </c>
       <c r="AI7" t="n">
         <v>2185184.4</v>
@@ -1405,7 +1405,7 @@
         <v>8</v>
       </c>
       <c r="K8" t="n">
-        <v>9.763333333333334</v>
+        <v>10.07</v>
       </c>
       <c r="L8" t="n">
         <v>3.033333333333333</v>
@@ -1448,7 +1448,7 @@
         <v>11.24888299217723</v>
       </c>
       <c r="AD8" t="n">
-        <v>-1.763333333333334</v>
+        <v>-2.07</v>
       </c>
       <c r="AE8" t="n">
         <v>5961.101261111111</v>
@@ -1460,7 +1460,7 @@
         <v>11.24888299217723</v>
       </c>
       <c r="AH8" t="n">
-        <v>1.485549658843899</v>
+        <v>1.178882992177233</v>
       </c>
       <c r="AI8" t="n">
         <v>2128943.1</v>
@@ -1540,7 +1540,7 @@
         <v>7.790322580645161</v>
       </c>
       <c r="K9" t="n">
-        <v>9.896666666666667</v>
+        <v>10.69666666666667</v>
       </c>
       <c r="L9" t="n">
         <v>7.933333333333333</v>
@@ -1583,7 +1583,7 @@
         <v>13.91723013647719</v>
       </c>
       <c r="AD9" t="n">
-        <v>-2.106344086021505</v>
+        <v>-2.906344086021506</v>
       </c>
       <c r="AE9" t="n">
         <v>6093.205149777778</v>
@@ -1595,7 +1595,7 @@
         <v>13.91723013647719</v>
       </c>
       <c r="AH9" t="n">
-        <v>4.02056346981052</v>
+        <v>3.22056346981052</v>
       </c>
       <c r="AI9" t="n">
         <v>2323049.3</v>
@@ -1675,7 +1675,7 @@
         <v>7.338709677419355</v>
       </c>
       <c r="K10" t="n">
-        <v>8.81</v>
+        <v>9.523333333333333</v>
       </c>
       <c r="L10" t="n">
         <v>1.1</v>
@@ -1718,7 +1718,7 @@
         <v>12.69099146058279</v>
       </c>
       <c r="AD10" t="n">
-        <v>-1.471290322580646</v>
+        <v>-2.184623655913978</v>
       </c>
       <c r="AE10" t="n">
         <v>5736.900974888889</v>
@@ -1730,7 +1730,7 @@
         <v>12.69099146058279</v>
       </c>
       <c r="AH10" t="n">
-        <v>3.88099146058279</v>
+        <v>3.167658127249457</v>
       </c>
       <c r="AI10" t="n">
         <v>2272050.6</v>
@@ -1812,7 +1812,7 @@
         <v>7.280555555555556</v>
       </c>
       <c r="K11" t="n">
-        <v>10.09</v>
+        <v>9.666666666666666</v>
       </c>
       <c r="L11" t="n">
         <v>4.8</v>
@@ -1855,7 +1855,7 @@
         <v>13.0042499150413</v>
       </c>
       <c r="AD11" t="n">
-        <v>-2.809444444444444</v>
+        <v>-2.38611111111111</v>
       </c>
       <c r="AE11" t="n">
         <v>6863.803933666666</v>
@@ -1867,7 +1867,7 @@
         <v>13.0042499150413</v>
       </c>
       <c r="AH11" t="n">
-        <v>2.914249915041299</v>
+        <v>3.337583248374633</v>
       </c>
       <c r="AI11" t="n">
         <v>2318883.3</v>
@@ -1949,7 +1949,7 @@
         <v>7.674731182795699</v>
       </c>
       <c r="K12" t="n">
-        <v>10.59333333333333</v>
+        <v>10.4</v>
       </c>
       <c r="L12" t="n">
         <v>3.033333333333333</v>
@@ -1992,7 +1992,7 @@
         <v>14.80433839943327</v>
       </c>
       <c r="AD12" t="n">
-        <v>-2.918602150537635</v>
+        <v>-2.725268817204301</v>
       </c>
       <c r="AE12" t="n">
         <v>6776.804489666667</v>
@@ -2004,7 +2004,7 @@
         <v>14.80433839943327</v>
       </c>
       <c r="AH12" t="n">
-        <v>4.211005066099936</v>
+        <v>4.40433839943327</v>
       </c>
       <c r="AI12" t="n">
         <v>2437481</v>
@@ -2226,7 +2226,7 @@
         <v>7.859999999999999</v>
       </c>
       <c r="L14" t="n">
-        <v>5.633333333333334</v>
+        <v>5.633333333333333</v>
       </c>
       <c r="M14" t="n">
         <v>59.79743333333334</v>
@@ -3870,7 +3870,7 @@
         <v>2.21</v>
       </c>
       <c r="L26" t="n">
-        <v>1.933333333333334</v>
+        <v>1.933333333333333</v>
       </c>
       <c r="M26" t="n">
         <v>64.45829999999999</v>
@@ -5103,7 +5103,7 @@
         <v>3.473333333333333</v>
       </c>
       <c r="L35" t="n">
-        <v>-0.3666666666666665</v>
+        <v>-0.3666666666666664</v>
       </c>
       <c r="M35" t="n">
         <v>70.42923333333333</v>
@@ -5511,7 +5511,7 @@
         <v>4.223655913978495</v>
       </c>
       <c r="K38" t="n">
-        <v>6.573333333333333</v>
+        <v>6.23</v>
       </c>
       <c r="L38" t="n">
         <v>-35.76666666666667</v>
@@ -5554,7 +5554,7 @@
         <v>12.31920706109511</v>
       </c>
       <c r="AD38" t="n">
-        <v>-2.349677419354839</v>
+        <v>-2.006344086021506</v>
       </c>
       <c r="AE38" t="n">
         <v>2226.407810666667</v>
@@ -5566,7 +5566,7 @@
         <v>12.31920706109511</v>
       </c>
       <c r="AH38" t="n">
-        <v>5.745873727761773</v>
+        <v>6.089207061095106</v>
       </c>
       <c r="AI38" t="n">
         <v>2661511.5</v>
@@ -8852,7 +8852,7 @@
         <v>5.25</v>
       </c>
       <c r="K61" t="n">
-        <v>3.12</v>
+        <v>3.116666666666667</v>
       </c>
       <c r="L61" t="n">
         <v>4.766666666666667</v>
@@ -8907,7 +8907,7 @@
         <v>10.65310701519588</v>
       </c>
       <c r="AD61" t="n">
-        <v>2.13</v>
+        <v>2.133333333333333</v>
       </c>
       <c r="AE61" t="n">
         <v>7333.314248222222</v>
@@ -8919,7 +8919,7 @@
         <v>10.65310701519588</v>
       </c>
       <c r="AH61" t="n">
-        <v>7.533107015195885</v>
+        <v>7.536440348529217</v>
       </c>
       <c r="AI61" t="inlineStr"/>
       <c r="AJ61" t="n">
@@ -8978,12 +8978,18 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
+      <c r="I62" t="n">
+        <v>4.3</v>
+      </c>
       <c r="J62" t="n">
         <v>5.25</v>
       </c>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
+      <c r="K62" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="L62" t="n">
+        <v>6.233333333333334</v>
+      </c>
       <c r="M62" t="n">
         <v>94.57384999999999</v>
       </c>
@@ -9033,7 +9039,9 @@
       <c r="AC62" t="n">
         <v>10.39133638585295</v>
       </c>
-      <c r="AD62" t="inlineStr"/>
+      <c r="AD62" t="n">
+        <v>1.32</v>
+      </c>
       <c r="AE62" t="n">
         <v>9767.271981833333</v>
       </c>
@@ -9043,7 +9051,9 @@
       <c r="AG62" t="n">
         <v>10.39133638585295</v>
       </c>
-      <c r="AH62" t="inlineStr"/>
+      <c r="AH62" t="n">
+        <v>6.461336385852945</v>
+      </c>
       <c r="AI62" t="inlineStr"/>
       <c r="AJ62" t="n">
         <v>34.5648235176878</v>
@@ -9101,10 +9111,16 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="n">
+        <v>4.3</v>
+      </c>
       <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
+      <c r="K63" t="n">
+        <v>4.635</v>
+      </c>
+      <c r="L63" t="n">
+        <v>6.7</v>
+      </c>
       <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="n">
@@ -9180,7 +9196,9 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
+      <c r="I64" t="n">
+        <v>4.3</v>
+      </c>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr"/>

</xml_diff>